<commit_message>
feat(balance): iteration 13 — master balance tables (docs/BALANCE.md generator + guard test); regenerate stale ENTITIES
</commit_message>
<xml_diff>
--- a/docs/ENTITIES.xlsx
+++ b/docs/ENTITIES.xlsx
@@ -171,7 +171,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>620 cr..680 cr</t>
+          <t>620000 cr..680000 cr</t>
         </is>
       </c>
     </row>
@@ -327,7 +327,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>380 cr..420 cr</t>
+          <t>380000 cr..420000 cr</t>
         </is>
       </c>
     </row>
@@ -383,12 +383,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>180 cr..220 cr</t>
+          <t>180000 cr..220000 cr</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>220 cr + 8 mat</t>
+          <t>220000 cr + 8 mat</t>
         </is>
       </c>
     </row>
@@ -444,12 +444,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>140 cr</t>
+          <t>140000 cr</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>90 cr + 4 mat</t>
+          <t>90000 cr + 4 mat</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -476,12 +476,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>180 cr</t>
+          <t>180000 cr</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>120 cr + 6 mat</t>
+          <t>120000 cr + 6 mat</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -527,7 +527,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>300 cr + 10 mat</t>
+          <t>300000 cr + 10 mat</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>450 cr + 15 mat</t>
+          <t>450000 cr + 15 mat</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>350 cr + 20 mat</t>
+          <t>350000 cr + 20 mat</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -578,12 +578,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>350 cr + 15 mat</t>
+          <t>350000 cr + 15 mat</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>— / building-workshop</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>building-medical-block</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>350000 cr + 20 mat</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>blueprint-medical-block / building-workshop</t>
         </is>
       </c>
     </row>
@@ -624,7 +641,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>150 cr</t>
+          <t>250000 cr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -646,7 +663,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>180 cr</t>
+          <t>300000 cr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -656,7 +673,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -668,7 +685,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>200 cr</t>
+          <t>250000 cr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -679,6 +696,72 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>staff-manager</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>400000 cr</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>staff-medic</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>280000 cr</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>building-medical-block</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>staff-repair-master</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>300000 cr</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>building-workshop</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -729,22 +812,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Interceptor</t>
+          <t>India aircraft</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -754,29 +837,29 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>30 cr</t>
+          <t>26000 cr</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>320000 cr..390000 cr</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gunship</t>
+          <t>British aircraft</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>125</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>0.92</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -791,86 +874,197 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>45 cr</t>
+          <t>42000 cr</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>900 cr..1100 cr</t>
+          <t>760000 cr..920000 cr</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aegis</t>
+          <t>PRC aircraft</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.05</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>60 cr</t>
+          <t>32000 cr</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1300 cr..1600 cr</t>
+          <t>520000 cr..620000 cr</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Yanlong</t>
+          <t>German aircraft</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>135</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>44000 cr</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>820000 cr..980000 cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>US aircraft</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>54000 cr</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1150000 cr..1400000 cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>French aircraft</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>50 cr</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>1000 cr..1300 cr</t>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1.05</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>34000 cr</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>580000 cr..700000 cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Japanese aircraft</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>56000 cr</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>620000 cr..740000 cr</t>
         </is>
       </c>
     </row>
@@ -911,7 +1105,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>40 cr + 1 mat</t>
+          <t>40000 cr + 1 mat</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -921,7 +1115,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>30 cr..50 cr</t>
+          <t>30000 cr..50000 cr</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1211,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>8000</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1064,7 +1258,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>12000</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1111,7 +1305,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>100000</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1158,7 +1352,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>16000</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1199,7 +1393,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>250 cr + 10 mat</t>
+          <t>250000 cr + 10 mat</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1299,7 +1493,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>blueprint-canister-cannon</t>
+          <t>blueprint-medical-block</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1319,34 +1513,61 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>weapon weapon-canister-cannon + production 200 cr</t>
+          <t>building building-medical-block</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>blueprint-canister-cannon</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3 sorties</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>building-laboratory + staff-scientist</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>weapon weapon-canister-cannon + production 200000 cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>blueprint-split-pulse-adaptation</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>alien</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>alien analysis</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>quarantine + lab</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>weapon weapon-split-pulse + production 250 cr</t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>weapon weapon-split-pulse + production 250000 cr</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(base): phase 1 — canonical building IDs (research-centre/production-works), typed lookups, save v18 migration
</commit_message>
<xml_diff>
--- a/docs/ENTITIES.xlsx
+++ b/docs/ENTITIES.xlsx
@@ -522,7 +522,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>building-laboratory</t>
+          <t>building-research-centre</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -539,7 +539,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>building-workshop</t>
+          <t>building-production-works</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>— / building-laboratory</t>
+          <t>— / building-research-centre</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>blueprint-safe-containment / building-workshop</t>
+          <t>blueprint-safe-containment / building-production-works</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>— / building-workshop</t>
+          <t>— / building-production-works</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>blueprint-medical-block / building-workshop</t>
+          <t>blueprint-medical-block / building-production-works</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>building-laboratory</t>
+          <t>building-research-centre</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>building-workshop</t>
+          <t>building-production-works</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>building-workshop</t>
+          <t>building-production-works</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>building-workshop + staff-engineer</t>
+          <t>building-production-works + staff-engineer</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>building-laboratory + staff-scientist</t>
+          <t>building-research-centre + staff-scientist</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>building-laboratory + staff-scientist</t>
+          <t>building-research-centre + staff-scientist</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>building-laboratory + staff-scientist</t>
+          <t>building-research-centre + staff-scientist</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>building-laboratory + staff-scientist</t>
+          <t>building-research-centre + staff-scientist</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">

</xml_diff>

<commit_message>
feat(base): Command Centre + Hangar as starter buildings with capability model (schema v19)
</commit_message>
<xml_diff>
--- a/docs/ENTITIES.xlsx
+++ b/docs/ENTITIES.xlsx
@@ -522,12 +522,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>building-research-centre</t>
+          <t>building-command-centre</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>300000 cr + 10 mat</t>
+          <t>400000 cr + 10 mat</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -539,66 +539,100 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>building-production-works</t>
+          <t>building-hangar</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>450000 cr + 15 mat</t>
+          <t>500000 cr + 20 mat</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>— / building-research-centre</t>
+          <t>— / —</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>building-quarantine-centre</t>
+          <t>building-research-centre</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>350000 cr + 20 mat</t>
+          <t>300000 cr + 10 mat</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>blueprint-safe-containment / building-production-works</t>
+          <t>— / —</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>building-trade-centre</t>
+          <t>building-production-works</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>350000 cr + 15 mat</t>
+          <t>450000 cr + 15 mat</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>— / building-production-works</t>
+          <t>— / building-research-centre</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>building-quarantine-centre</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>350000 cr + 20 mat</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>blueprint-safe-containment / building-production-works</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>building-trade-centre</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>350000 cr + 15 mat</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>— / building-production-works</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>building-medical-block</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>350000 cr + 20 mat</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>blueprint-medical-block / building-production-works</t>
         </is>

</xml_diff>

<commit_message>
docs(weapons): E1b — ENTITIES generator covers full arsenal, INDEX.md, localize() helper, drift guard test
</commit_message>
<xml_diff>
--- a/docs/ENTITIES.xlsx
+++ b/docs/ENTITIES.xlsx
@@ -12,6 +12,12 @@
     <sheet name="Equipment" sheetId="8" r:id="rId8"/>
     <sheet name="Research" sheetId="9" r:id="rId9"/>
     <sheet name="Market blueprints" sheetId="10" r:id="rId10"/>
+    <sheet name="Weapon families" sheetId="11" r:id="rId11"/>
+    <sheet name="Weapon Marks" sheetId="12" r:id="rId12"/>
+    <sheet name="Auxiliary" sheetId="13" r:id="rId13"/>
+    <sheet name="Modules" sheetId="14" r:id="rId14"/>
+    <sheet name="Ammunition" sheetId="15" r:id="rId15"/>
+    <sheet name="Aircraft loadouts" sheetId="16" r:id="rId16"/>
   </sheets>
 </workbook>
 </file>
@@ -396,6 +402,2989 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Tech family</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Damage</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Shots/s</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Projectiles</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Penetration</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Acquisition</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Marks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>weapon-autocannon</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>human-kinetic</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>620</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>single-target</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Mk2, Mk3, Mk4, Mk5, Mk6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>weapon-heavy-autocannon</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>human-kinetic</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>560</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>single-target</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Mk2, Mk3, Mk4, Mk5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>weapon-gatling-gun</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>human-kinetic</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>650</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>single-target</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Mk2, Mk3, Mk4, Mk5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>weapon-scatter-cannon</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>human-kinetic</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>520</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>single-target</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Mk2, Mk3, Mk4, Mk5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>weapon-railgun</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>human-kinetic</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>all-targets</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Mk2, Mk3, Mk4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>weapon-flak-cannon</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>human-kinetic</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>single-target</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Mk2, Mk3, Mk4, Mk5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>weapon-pulse-laser</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>hybrid-laser</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1250</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>single-target</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Mk2, Mk3, Mk4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>weapon-plasma-machine-gun</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>hybrid-plasma</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>760</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>single-target</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Mk2, Mk3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>weapon-plasma-cannon</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>hybrid-plasma</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>520</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>single-target</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Mk2, Mk3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>weapon-disintegration-lance</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>alien</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>alien</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>all-targets</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>alien-recovery</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>weapon-plasma-orb-projector</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>alien</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>alien</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0.65</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>all-targets</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>alien-recovery</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>weapon-singularity-projector</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>alien</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>alien</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>all-targets</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>alien-recovery</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Mark</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Research cost</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Production cost</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Overrides</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>weapon-autocannon-mk-2</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>100000 cr</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>50000 cr + 5 mat</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>damage=12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>weapon-autocannon-mk-3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>160000 cr</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>80000 cr + 8 mat</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>shotsPerSecond=6.5, spreadDegrees=1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>weapon-autocannon-mk-4</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>240000 cr</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>120000 cr + 12 mat</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>damage=15, projectileSpeed=660</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>weapon-autocannon-mk-5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>360000 cr</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>180000 cr + 18 mat</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>damage=18, shotsPerSecond=7, spreadDegrees=1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>weapon-autocannon-mk-6</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>520000 cr</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>280000 cr + 26 mat</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>damage=22, shotsPerSecond=7.5, spreadDegrees=1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>weapon-heavy-autocannon-mk-2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>140000 cr</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>90000 cr + 9 mat</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>shotsPerSecond=2.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>weapon-heavy-autocannon-mk-3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>220000 cr</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>130000 cr + 13 mat</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>damage=30</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>weapon-heavy-autocannon-mk-4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>340000 cr</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>190000 cr + 19 mat</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>damage=34, shotsPerSecond=2.8, spreadDegrees=1.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>weapon-heavy-autocannon-mk-5</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>480000 cr</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>270000 cr + 25 mat</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>damage=40, shotsPerSecond=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>weapon-gatling-gun-mk-2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>140000 cr</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>90000 cr + 9 mat</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>shotsPerSecond=10</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>weapon-gatling-gun-mk-3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>220000 cr</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>140000 cr + 14 mat</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>spreadDegrees=3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>weapon-gatling-gun-mk-4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>340000 cr</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>200000 cr + 20 mat</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>damage=8.5, shotsPerSecond=10.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>weapon-gatling-gun-mk-5</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>480000 cr</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>290000 cr + 27 mat</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>damage=10, shotsPerSecond=12</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>weapon-scatter-cannon-mk-2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>130000 cr</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>80000 cr + 8 mat</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>damage=9</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>weapon-scatter-cannon-mk-3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>200000 cr</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>120000 cr + 12 mat</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>damage=10, projectileCount=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>weapon-scatter-cannon-mk-4</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>300000 cr</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>180000 cr + 18 mat</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>damage=11, projectileCount=8, projectileSpeed=540</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>weapon-scatter-cannon-mk-5</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>440000 cr</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>250000 cr + 24 mat</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>damage=12, projectileCount=8, projectileSpeed=560</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>weapon-railgun-mk-2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>240000 cr</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>160000 cr + 16 mat</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>shotsPerSecond=0.85</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>weapon-railgun-mk-3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>380000 cr</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>240000 cr + 23 mat</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>damage=60, projectileSpeed=1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>weapon-railgun-mk-4</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>560000 cr</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>350000 cr + 32 mat</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>damage=72, shotsPerSecond=0.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>weapon-flak-cannon-mk-2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>160000 cr</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>100000 cr + 10 mat</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>damage=18</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>weapon-flak-cannon-mk-3</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>240000 cr</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>150000 cr + 15 mat</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>damage=20</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>weapon-flak-cannon-mk-4</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>360000 cr</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>210000 cr + 21 mat</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>damage=23, projectileSpeed=540</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>weapon-flak-cannon-mk-5</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>500000 cr</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>290000 cr + 28 mat</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>damage=27, projectileSpeed=560</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>weapon-pulse-laser-mk-2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>320000 cr</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>200000 cr + 18 mat</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>damage=24, shotsPerSecond=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>weapon-pulse-laser-mk-3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>480000 cr</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>300000 cr + 26 mat</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>damage=28, spreadDegrees=0.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>weapon-pulse-laser-mk-4</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>680000 cr</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>440000 cr + 36 mat</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>damage=34, shotsPerSecond=7.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>weapon-plasma-machine-gun-mk-2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>640000 cr</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>420000 cr + 34 mat</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>damage=34, shotsPerSecond=8</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>weapon-plasma-machine-gun-mk-3</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>940000 cr</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>620000 cr + 48 mat</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>damage=40, shotsPerSecond=8.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>weapon-plasma-cannon-mk-2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>700000 cr</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>460000 cr + 38 mat</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>damage=104</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>weapon-plasma-cannon-mk-3</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1040000 cr</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>700000 cr + 54 mat</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>damage=120, shotsPerSecond=1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Auxiliary</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Ammo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Charges</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Damage</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Radius</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Stun s</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>aux-rocket-pod</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>rocket</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>consumable-rocket</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>3..12</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>aux-homing-missile-rack</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>homing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>consumable-homing-missile</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4..10</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>aux-heavy-torpedo-launcher</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>torpedo</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>consumable-heavy-torpedo</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1..4</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>aux-cluster-missile-pod</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cluster</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>consumable-cluster-missile</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2..6</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>aux-ukrainian-drone-swarm</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>drone</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>consumable-ukrainian-attack-drone</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>50..100</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>aux-stun-module</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>stun</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0..0</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Effect</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>module-energy-shield</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Adds a regenerating damage buffer that absorbs incoming damage before armour.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>module-directional-energy-shield</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Stronger shield against the forward arc, little protection from the rear.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>module-dash</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>dash</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Enables a short high-speed directional dash with a cooldown.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>module-targeting-computer</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>targeting</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Improves primary-weapon accuracy and precision damage.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>module-repair-nanobots</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Slowly restores armour during flight after avoiding damage.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>module-reflector-field</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>reflector</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Periodically reflects a fraction of eligible hostile projectiles back.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Ammo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Weight/unit</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Used by</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>consumable-rocket</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>40 cr</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>aux-rocket-pod</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>consumable-homing-missile</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>70 cr</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>aux-homing-missile-rack</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>consumable-heavy-torpedo</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>120 cr</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>aux-heavy-torpedo-launcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>consumable-cluster-missile</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>100 cr</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>aux-cluster-missile-pod</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>consumable-ukrainian-attack-drone</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0.06</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>6 cr</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>aux-ukrainian-drone-swarm</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Aircraft</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Armour</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Speed x</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>dmg/fire/acc x</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>1° slots</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Hardpoints</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Reactor</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Marks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>aircraft-india</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>workhorse</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.95 / 1 / 1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Mk2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>aircraft-britain</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>bruiser</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.92</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.15 / 0.95 / 1.05</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Mk2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>aircraft-prc</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>interceptor</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.05 / 1.1 / 1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Mk2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>aircraft-germany</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>precision</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.1 / 1 / 1.1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Mk2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>aircraft-usa</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>gunship</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.25 / 0.95 / 0.95</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Mk2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>aircraft-france</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>duelist</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.05 / 1.05 / 1.1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Mk2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>aircraft-japan</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>glass-cannon</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.45 / 1.05 / 1.1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Mk2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>

</xml_diff>

<commit_message>
feat(weapons): E2b-3b — aircraft Mark II/III pipeline (Mark III data, mark applied on upgrade production)
</commit_message>
<xml_diff>
--- a/docs/ENTITIES.xlsx
+++ b/docs/ENTITIES.xlsx
@@ -3065,7 +3065,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Mk2</t>
+          <t>Mk2, Mk3</t>
         </is>
       </c>
     </row>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Mk2</t>
+          <t>Mk2, Mk3</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Mk2</t>
+          <t>Mk2, Mk3</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Mk2</t>
+          <t>Mk2, Mk3</t>
         </is>
       </c>
     </row>
@@ -3273,7 +3273,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Mk2</t>
+          <t>Mk2, Mk3</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Mk2</t>
+          <t>Mk2, Mk3</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Mk2</t>
+          <t>Mk2, Mk3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(weapons): E3.4b — flare/decoy launcher attracts and absorbs enemy homing missiles
</commit_message>
<xml_diff>
--- a/docs/ENTITIES.xlsx
+++ b/docs/ENTITIES.xlsx
@@ -2553,6 +2553,63 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>aux-flare-decoy-launcher</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>decoy</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>consumable-flare-decoy</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>3..6</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>research-production</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -2958,6 +3015,28 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>consumable-flare-decoy</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>25 cr</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>aux-flare-decoy-launcher</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>